<commit_message>
Map Stolen Bell's Toast job titles; add Busser as a support role
- config/tipout.yaml maps the real titles: Bartender/Lead Bartender ->
  Bartender, Server/Lead Server -> Server, Host, Barback, Busser, and
  Kitchen All Rounder/Chef de Partie/Sous Chef/Chef -> Kitchen.
- Busser shares the support cut. The support rate is 2.25% when two or
  more different support roles worked, 1.5% for one (as the engine
  already computed); the skill text, Cash Out form formula and its role
  dropdown now say the same.
- Demo restaurant uses the real kitchen titles and a weekend Busser.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015jcTPXYQVoMy2BAsKbkHbq
</commit_message>
<xml_diff>
--- a/skills/stolen-bell-tipout/forms/CashOut_Form.xlsx
+++ b/skills/stolen-bell-tipout/forms/CashOut_Form.xlsx
@@ -574,13 +574,13 @@
           <t>Date</t>
         </is>
       </c>
-      <c r="B4" s="24" t="n"/>
+      <c r="B4" s="35" t="n"/>
       <c r="D4" s="23" t="inlineStr">
         <is>
           <t>Service</t>
         </is>
       </c>
-      <c r="E4" s="24" t="n"/>
+      <c r="E4" s="35" t="n"/>
     </row>
     <row r="5" ht="15" customHeight="1" s="20">
       <c r="A5" s="23" t="inlineStr">
@@ -588,7 +588,7 @@
           <t>Completed by</t>
         </is>
       </c>
-      <c r="B5" s="24" t="n"/>
+      <c r="B5" s="35" t="n"/>
     </row>
     <row r="7" ht="15" customHeight="1" s="20">
       <c r="A7" s="25" t="inlineStr">
@@ -681,7 +681,7 @@
           <t>Kitchen — 10% of gross FOOD sales</t>
         </is>
       </c>
-      <c r="B19" s="29">
+      <c r="B19" s="38">
         <f>0.1*B10</f>
         <v/>
       </c>
@@ -694,11 +694,11 @@
     <row r="20" ht="15" customHeight="1" s="20">
       <c r="A20" s="23" t="inlineStr">
         <is>
-          <t>Support rate  (auto: 1.5% Host or Barback, 2.25% both)</t>
+          <t>Support rate  (auto: 1.5% one role, 2.25% two or more)</t>
         </is>
       </c>
       <c r="B20" s="30">
-        <f>IF(AND(COUNTIFS($E$23:$E$25,"Host",$C$23:$C$25,"&gt;0")&gt;0,COUNTIFS($E$23:$E$25,"Barback",$C$23:$C$25,"&gt;0")&gt;0),0.0225,IF(COUNTIFS($E$23:$E$25,"Host",$C$23:$C$25,"&gt;0")+COUNTIFS($E$23:$E$25,"Barback",$C$23:$C$25,"&gt;0")&gt;0,0.015,0))</f>
+        <f>IF((COUNTIFS($E$23:$E$25,"Host",$C$23:$C$25,"&gt;0")&gt;0)+(COUNTIFS($E$23:$E$25,"Barback",$C$23:$C$25,"&gt;0")&gt;0)+(COUNTIFS($E$23:$E$25,"Busser",$C$23:$C$25,"&gt;0")&gt;0)&gt;=2,0.0225,IF((COUNTIFS($E$23:$E$25,"Host",$C$23:$C$25,"&gt;0")&gt;0)+(COUNTIFS($E$23:$E$25,"Barback",$C$23:$C$25,"&gt;0")&gt;0)+(COUNTIFS($E$23:$E$25,"Busser",$C$23:$C$25,"&gt;0")&gt;0)=1,0.015,0))</f>
         <v/>
       </c>
     </row>
@@ -714,17 +714,17 @@
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="20">
-      <c r="B22" s="31" t="inlineStr">
+      <c r="B22" s="32" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C22" s="31" t="inlineStr">
+      <c r="C22" s="32" t="inlineStr">
         <is>
           <t>Hours</t>
         </is>
       </c>
-      <c r="D22" s="31" t="inlineStr">
+      <c r="D22" s="32" t="inlineStr">
         <is>
           <t>Payout</t>
         </is>
@@ -736,28 +736,28 @@
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="20">
-      <c r="A23" s="33" t="inlineStr">
+      <c r="A23" s="36" t="inlineStr">
         <is>
           <t>Support 1</t>
         </is>
       </c>
-      <c r="B23" s="24" t="n"/>
-      <c r="C23" s="34" t="n"/>
-      <c r="D23" s="29">
+      <c r="B23" s="35" t="n"/>
+      <c r="C23" s="37" t="n"/>
+      <c r="D23" s="38">
         <f>IF(SUM($C$23:$C$25)&gt;0,$B$21*C23/SUM($C$23:$C$25),0)</f>
         <v/>
       </c>
       <c r="E23" s="35" t="n"/>
     </row>
     <row r="24" ht="15" customHeight="1" s="20">
-      <c r="A24" s="33" t="inlineStr">
+      <c r="A24" s="36" t="inlineStr">
         <is>
           <t>Support 2  (if any)</t>
         </is>
       </c>
-      <c r="B24" s="24" t="n"/>
-      <c r="C24" s="34" t="n"/>
-      <c r="D24" s="29">
+      <c r="B24" s="35" t="n"/>
+      <c r="C24" s="37" t="n"/>
+      <c r="D24" s="38">
         <f>IF(SUM($C$23:$C$25)&gt;0,$B$21*C24/SUM($C$23:$C$25),0)</f>
         <v/>
       </c>
@@ -833,13 +833,13 @@
       <c r="A30" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="B30" s="24" t="n"/>
-      <c r="C30" s="34" t="n"/>
+      <c r="B30" s="35" t="n"/>
+      <c r="C30" s="37" t="n"/>
       <c r="D30" s="38">
         <f>IF(AND(C30&gt;0,$C$40&gt;0),$B$26/$C$40,"")</f>
         <v/>
       </c>
-      <c r="E30" s="29">
+      <c r="E30" s="38">
         <f>IF($C$40&gt;0,$B$26*C30/$C$40,0)</f>
         <v/>
       </c>
@@ -848,13 +848,13 @@
       <c r="A31" s="40" t="n">
         <v>2</v>
       </c>
-      <c r="B31" s="24" t="n"/>
-      <c r="C31" s="34" t="n"/>
+      <c r="B31" s="35" t="n"/>
+      <c r="C31" s="37" t="n"/>
       <c r="D31" s="38">
         <f>IF(AND(C31&gt;0,$C$40&gt;0),$B$26/$C$40,"")</f>
         <v/>
       </c>
-      <c r="E31" s="29">
+      <c r="E31" s="38">
         <f>IF($C$40&gt;0,$B$26*C31/$C$40,0)</f>
         <v/>
       </c>
@@ -863,13 +863,13 @@
       <c r="A32" s="40" t="n">
         <v>3</v>
       </c>
-      <c r="B32" s="24" t="n"/>
-      <c r="C32" s="34" t="n"/>
+      <c r="B32" s="35" t="n"/>
+      <c r="C32" s="37" t="n"/>
       <c r="D32" s="38">
         <f>IF(AND(C32&gt;0,$C$40&gt;0),$B$26/$C$40,"")</f>
         <v/>
       </c>
-      <c r="E32" s="29">
+      <c r="E32" s="38">
         <f>IF($C$40&gt;0,$B$26*C32/$C$40,0)</f>
         <v/>
       </c>
@@ -878,13 +878,13 @@
       <c r="A33" s="40" t="n">
         <v>4</v>
       </c>
-      <c r="B33" s="24" t="n"/>
-      <c r="C33" s="34" t="n"/>
+      <c r="B33" s="35" t="n"/>
+      <c r="C33" s="37" t="n"/>
       <c r="D33" s="38">
         <f>IF(AND(C33&gt;0,$C$40&gt;0),$B$26/$C$40,"")</f>
         <v/>
       </c>
-      <c r="E33" s="29">
+      <c r="E33" s="38">
         <f>IF($C$40&gt;0,$B$26*C33/$C$40,0)</f>
         <v/>
       </c>
@@ -893,13 +893,13 @@
       <c r="A34" s="40" t="n">
         <v>5</v>
       </c>
-      <c r="B34" s="24" t="n"/>
-      <c r="C34" s="34" t="n"/>
+      <c r="B34" s="35" t="n"/>
+      <c r="C34" s="37" t="n"/>
       <c r="D34" s="38">
         <f>IF(AND(C34&gt;0,$C$40&gt;0),$B$26/$C$40,"")</f>
         <v/>
       </c>
-      <c r="E34" s="29">
+      <c r="E34" s="38">
         <f>IF($C$40&gt;0,$B$26*C34/$C$40,0)</f>
         <v/>
       </c>
@@ -908,13 +908,13 @@
       <c r="A35" s="40" t="n">
         <v>6</v>
       </c>
-      <c r="B35" s="24" t="n"/>
-      <c r="C35" s="34" t="n"/>
+      <c r="B35" s="35" t="n"/>
+      <c r="C35" s="37" t="n"/>
       <c r="D35" s="38">
         <f>IF(AND(C35&gt;0,$C$40&gt;0),$B$26/$C$40,"")</f>
         <v/>
       </c>
-      <c r="E35" s="29">
+      <c r="E35" s="38">
         <f>IF($C$40&gt;0,$B$26*C35/$C$40,0)</f>
         <v/>
       </c>
@@ -923,13 +923,13 @@
       <c r="A36" s="40" t="n">
         <v>7</v>
       </c>
-      <c r="B36" s="24" t="n"/>
-      <c r="C36" s="34" t="n"/>
+      <c r="B36" s="35" t="n"/>
+      <c r="C36" s="37" t="n"/>
       <c r="D36" s="38">
         <f>IF(AND(C36&gt;0,$C$40&gt;0),$B$26/$C$40,"")</f>
         <v/>
       </c>
-      <c r="E36" s="29">
+      <c r="E36" s="38">
         <f>IF($C$40&gt;0,$B$26*C36/$C$40,0)</f>
         <v/>
       </c>
@@ -938,13 +938,13 @@
       <c r="A37" s="40" t="n">
         <v>8</v>
       </c>
-      <c r="B37" s="24" t="n"/>
-      <c r="C37" s="34" t="n"/>
+      <c r="B37" s="35" t="n"/>
+      <c r="C37" s="37" t="n"/>
       <c r="D37" s="38">
         <f>IF(AND(C37&gt;0,$C$40&gt;0),$B$26/$C$40,"")</f>
         <v/>
       </c>
-      <c r="E37" s="29">
+      <c r="E37" s="38">
         <f>IF($C$40&gt;0,$B$26*C37/$C$40,0)</f>
         <v/>
       </c>
@@ -953,13 +953,13 @@
       <c r="A38" s="40" t="n">
         <v>9</v>
       </c>
-      <c r="B38" s="24" t="n"/>
-      <c r="C38" s="34" t="n"/>
+      <c r="B38" s="35" t="n"/>
+      <c r="C38" s="37" t="n"/>
       <c r="D38" s="38">
         <f>IF(AND(C38&gt;0,$C$40&gt;0),$B$26/$C$40,"")</f>
         <v/>
       </c>
-      <c r="E38" s="29">
+      <c r="E38" s="38">
         <f>IF($C$40&gt;0,$B$26*C38/$C$40,0)</f>
         <v/>
       </c>
@@ -968,13 +968,13 @@
       <c r="A39" s="40" t="n">
         <v>10</v>
       </c>
-      <c r="B39" s="24" t="n"/>
-      <c r="C39" s="34" t="n"/>
+      <c r="B39" s="35" t="n"/>
+      <c r="C39" s="37" t="n"/>
       <c r="D39" s="38">
         <f>IF(AND(C39&gt;0,$C$40&gt;0),$B$26/$C$40,"")</f>
         <v/>
       </c>
-      <c r="E39" s="29">
+      <c r="E39" s="38">
         <f>IF($C$40&gt;0,$B$26*C39/$C$40,0)</f>
         <v/>
       </c>
@@ -1007,7 +1007,7 @@
           <t>Kitchen + Support + Bar/Servers</t>
         </is>
       </c>
-      <c r="B43" s="29">
+      <c r="B43" s="38">
         <f>B19+B21+E40</f>
         <v/>
       </c>
@@ -1018,7 +1018,7 @@
           <t>Total Tips (pool)</t>
         </is>
       </c>
-      <c r="B44" s="29">
+      <c r="B44" s="38">
         <f>B16</f>
         <v/>
       </c>
@@ -1057,7 +1057,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation sqref="E23:E25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Host,Barback"</formula1>
+      <formula1>"Host,Barback,Busser"</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -1102,7 +1102,7 @@
           <t>Date</t>
         </is>
       </c>
-      <c r="B4" s="24" t="inlineStr">
+      <c r="B4" s="35" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>
@@ -1112,7 +1112,7 @@
           <t>Service</t>
         </is>
       </c>
-      <c r="E4" s="24" t="inlineStr">
+      <c r="E4" s="35" t="inlineStr">
         <is>
           <t>Dinner</t>
         </is>
@@ -1124,7 +1124,7 @@
           <t>Completed by</t>
         </is>
       </c>
-      <c r="B5" s="24" t="inlineStr">
+      <c r="B5" s="35" t="inlineStr">
         <is>
           <t>S. Thornton</t>
         </is>
@@ -1233,7 +1233,7 @@
           <t>Kitchen — 10% of gross FOOD sales</t>
         </is>
       </c>
-      <c r="B19" s="29">
+      <c r="B19" s="38">
         <f>0.1*B10</f>
         <v/>
       </c>
@@ -1246,11 +1246,11 @@
     <row r="20" ht="15" customHeight="1" s="20">
       <c r="A20" s="23" t="inlineStr">
         <is>
-          <t>Support rate  (auto: 1.5% Host or Barback, 2.25% both)</t>
+          <t>Support rate  (auto: 1.5% one role, 2.25% two or more)</t>
         </is>
       </c>
       <c r="B20" s="30">
-        <f>IF(AND(COUNTIFS($E$23:$E$25,"Host",$C$23:$C$25,"&gt;0")&gt;0,COUNTIFS($E$23:$E$25,"Barback",$C$23:$C$25,"&gt;0")&gt;0),0.0225,IF(COUNTIFS($E$23:$E$25,"Host",$C$23:$C$25,"&gt;0")+COUNTIFS($E$23:$E$25,"Barback",$C$23:$C$25,"&gt;0")&gt;0,0.015,0))</f>
+        <f>IF((COUNTIFS($E$23:$E$25,"Host",$C$23:$C$25,"&gt;0")&gt;0)+(COUNTIFS($E$23:$E$25,"Barback",$C$23:$C$25,"&gt;0")&gt;0)+(COUNTIFS($E$23:$E$25,"Busser",$C$23:$C$25,"&gt;0")&gt;0)&gt;=2,0.0225,IF((COUNTIFS($E$23:$E$25,"Host",$C$23:$C$25,"&gt;0")&gt;0)+(COUNTIFS($E$23:$E$25,"Barback",$C$23:$C$25,"&gt;0")&gt;0)+(COUNTIFS($E$23:$E$25,"Busser",$C$23:$C$25,"&gt;0")&gt;0)=1,0.015,0))</f>
         <v/>
       </c>
     </row>
@@ -1266,17 +1266,17 @@
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="20">
-      <c r="B22" s="31" t="inlineStr">
+      <c r="B22" s="32" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C22" s="31" t="inlineStr">
+      <c r="C22" s="32" t="inlineStr">
         <is>
           <t>Hours</t>
         </is>
       </c>
-      <c r="D22" s="31" t="inlineStr">
+      <c r="D22" s="32" t="inlineStr">
         <is>
           <t>Payout</t>
         </is>
@@ -1288,20 +1288,20 @@
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="20">
-      <c r="A23" s="33" t="inlineStr">
+      <c r="A23" s="36" t="inlineStr">
         <is>
           <t>Support 1</t>
         </is>
       </c>
-      <c r="B23" s="24" t="inlineStr">
+      <c r="B23" s="35" t="inlineStr">
         <is>
           <t>Priya</t>
         </is>
       </c>
-      <c r="C23" s="34" t="n">
+      <c r="C23" s="37" t="n">
         <v>5</v>
       </c>
-      <c r="D23" s="29">
+      <c r="D23" s="38">
         <f>IF(SUM($C$23:$C$25)&gt;0,$B$21*C23/SUM($C$23:$C$25),0)</f>
         <v/>
       </c>
@@ -1312,20 +1312,20 @@
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="20">
-      <c r="A24" s="33" t="inlineStr">
+      <c r="A24" s="36" t="inlineStr">
         <is>
           <t>Support 2  (if any)</t>
         </is>
       </c>
-      <c r="B24" s="24" t="inlineStr">
+      <c r="B24" s="35" t="inlineStr">
         <is>
           <t>Tomas</t>
         </is>
       </c>
-      <c r="C24" s="34" t="n">
+      <c r="C24" s="37" t="n">
         <v>4</v>
       </c>
-      <c r="D24" s="29">
+      <c r="D24" s="38">
         <f>IF(SUM($C$23:$C$25)&gt;0,$B$21*C24/SUM($C$23:$C$25),0)</f>
         <v/>
       </c>
@@ -1405,19 +1405,19 @@
       <c r="A30" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="B30" s="24" t="inlineStr">
+      <c r="B30" s="35" t="inlineStr">
         <is>
           <t>Mara</t>
         </is>
       </c>
-      <c r="C30" s="34" t="n">
+      <c r="C30" s="37" t="n">
         <v>8</v>
       </c>
       <c r="D30" s="38">
         <f>IF(AND(C30&gt;0,$C$40&gt;0),$B$26/$C$40,"")</f>
         <v/>
       </c>
-      <c r="E30" s="29">
+      <c r="E30" s="38">
         <f>IF($C$40&gt;0,$B$26*C30/$C$40,0)</f>
         <v/>
       </c>
@@ -1426,19 +1426,19 @@
       <c r="A31" s="40" t="n">
         <v>2</v>
       </c>
-      <c r="B31" s="24" t="inlineStr">
+      <c r="B31" s="35" t="inlineStr">
         <is>
           <t>Devon</t>
         </is>
       </c>
-      <c r="C31" s="34" t="n">
+      <c r="C31" s="37" t="n">
         <v>6</v>
       </c>
       <c r="D31" s="38">
         <f>IF(AND(C31&gt;0,$C$40&gt;0),$B$26/$C$40,"")</f>
         <v/>
       </c>
-      <c r="E31" s="29">
+      <c r="E31" s="38">
         <f>IF($C$40&gt;0,$B$26*C31/$C$40,0)</f>
         <v/>
       </c>
@@ -1447,19 +1447,19 @@
       <c r="A32" s="40" t="n">
         <v>3</v>
       </c>
-      <c r="B32" s="24" t="inlineStr">
+      <c r="B32" s="35" t="inlineStr">
         <is>
           <t>Sam</t>
         </is>
       </c>
-      <c r="C32" s="34" t="n">
+      <c r="C32" s="37" t="n">
         <v>5</v>
       </c>
       <c r="D32" s="38">
         <f>IF(AND(C32&gt;0,$C$40&gt;0),$B$26/$C$40,"")</f>
         <v/>
       </c>
-      <c r="E32" s="29">
+      <c r="E32" s="38">
         <f>IF($C$40&gt;0,$B$26*C32/$C$40,0)</f>
         <v/>
       </c>
@@ -1468,13 +1468,13 @@
       <c r="A33" s="40" t="n">
         <v>4</v>
       </c>
-      <c r="B33" s="24" t="n"/>
-      <c r="C33" s="34" t="n"/>
+      <c r="B33" s="35" t="n"/>
+      <c r="C33" s="37" t="n"/>
       <c r="D33" s="38">
         <f>IF(AND(C33&gt;0,$C$40&gt;0),$B$26/$C$40,"")</f>
         <v/>
       </c>
-      <c r="E33" s="29">
+      <c r="E33" s="38">
         <f>IF($C$40&gt;0,$B$26*C33/$C$40,0)</f>
         <v/>
       </c>
@@ -1483,13 +1483,13 @@
       <c r="A34" s="40" t="n">
         <v>5</v>
       </c>
-      <c r="B34" s="24" t="n"/>
-      <c r="C34" s="34" t="n"/>
+      <c r="B34" s="35" t="n"/>
+      <c r="C34" s="37" t="n"/>
       <c r="D34" s="38">
         <f>IF(AND(C34&gt;0,$C$40&gt;0),$B$26/$C$40,"")</f>
         <v/>
       </c>
-      <c r="E34" s="29">
+      <c r="E34" s="38">
         <f>IF($C$40&gt;0,$B$26*C34/$C$40,0)</f>
         <v/>
       </c>
@@ -1498,13 +1498,13 @@
       <c r="A35" s="40" t="n">
         <v>6</v>
       </c>
-      <c r="B35" s="24" t="n"/>
-      <c r="C35" s="34" t="n"/>
+      <c r="B35" s="35" t="n"/>
+      <c r="C35" s="37" t="n"/>
       <c r="D35" s="38">
         <f>IF(AND(C35&gt;0,$C$40&gt;0),$B$26/$C$40,"")</f>
         <v/>
       </c>
-      <c r="E35" s="29">
+      <c r="E35" s="38">
         <f>IF($C$40&gt;0,$B$26*C35/$C$40,0)</f>
         <v/>
       </c>
@@ -1513,13 +1513,13 @@
       <c r="A36" s="40" t="n">
         <v>7</v>
       </c>
-      <c r="B36" s="24" t="n"/>
-      <c r="C36" s="34" t="n"/>
+      <c r="B36" s="35" t="n"/>
+      <c r="C36" s="37" t="n"/>
       <c r="D36" s="38">
         <f>IF(AND(C36&gt;0,$C$40&gt;0),$B$26/$C$40,"")</f>
         <v/>
       </c>
-      <c r="E36" s="29">
+      <c r="E36" s="38">
         <f>IF($C$40&gt;0,$B$26*C36/$C$40,0)</f>
         <v/>
       </c>
@@ -1528,13 +1528,13 @@
       <c r="A37" s="40" t="n">
         <v>8</v>
       </c>
-      <c r="B37" s="24" t="n"/>
-      <c r="C37" s="34" t="n"/>
+      <c r="B37" s="35" t="n"/>
+      <c r="C37" s="37" t="n"/>
       <c r="D37" s="38">
         <f>IF(AND(C37&gt;0,$C$40&gt;0),$B$26/$C$40,"")</f>
         <v/>
       </c>
-      <c r="E37" s="29">
+      <c r="E37" s="38">
         <f>IF($C$40&gt;0,$B$26*C37/$C$40,0)</f>
         <v/>
       </c>
@@ -1543,13 +1543,13 @@
       <c r="A38" s="40" t="n">
         <v>9</v>
       </c>
-      <c r="B38" s="24" t="n"/>
-      <c r="C38" s="34" t="n"/>
+      <c r="B38" s="35" t="n"/>
+      <c r="C38" s="37" t="n"/>
       <c r="D38" s="38">
         <f>IF(AND(C38&gt;0,$C$40&gt;0),$B$26/$C$40,"")</f>
         <v/>
       </c>
-      <c r="E38" s="29">
+      <c r="E38" s="38">
         <f>IF($C$40&gt;0,$B$26*C38/$C$40,0)</f>
         <v/>
       </c>
@@ -1558,13 +1558,13 @@
       <c r="A39" s="40" t="n">
         <v>10</v>
       </c>
-      <c r="B39" s="24" t="n"/>
-      <c r="C39" s="34" t="n"/>
+      <c r="B39" s="35" t="n"/>
+      <c r="C39" s="37" t="n"/>
       <c r="D39" s="38">
         <f>IF(AND(C39&gt;0,$C$40&gt;0),$B$26/$C$40,"")</f>
         <v/>
       </c>
-      <c r="E39" s="29">
+      <c r="E39" s="38">
         <f>IF($C$40&gt;0,$B$26*C39/$C$40,0)</f>
         <v/>
       </c>
@@ -1597,7 +1597,7 @@
           <t>Kitchen + Support + Bar/Servers</t>
         </is>
       </c>
-      <c r="B43" s="29">
+      <c r="B43" s="38">
         <f>B19+B21+E40</f>
         <v/>
       </c>
@@ -1608,7 +1608,7 @@
           <t>Total Tips (pool)</t>
         </is>
       </c>
-      <c r="B44" s="29">
+      <c r="B44" s="38">
         <f>B16</f>
         <v/>
       </c>
@@ -1647,7 +1647,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation sqref="E23:E25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Host,Barback"</formula1>
+      <formula1>"Host,Barback,Busser"</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>

<commit_message>
Map all Stolen Bell roles; add Runner support role and catch-all for other jobs
- Not tipped: Chef OFFICE, Admin, General Manager, Owner, Lead Bartender ADMIN.
- Kitchen: Chef, Sous Chef, Chef de Partie, Kitchen All Rounder, Cook.
- Support: Host, Barback, Busser, Runner (Runner added to the engine,
  support-rate rule and Cash Out form dropdown/formula).
- New otherJobs setting: any job not listed shares the bar/server
  remainder (Stolen Bell's rule), and each run names the jobs handled
  that way. 'stop' keeps the old behaviour.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015jcTPXYQVoMy2BAsKbkHbq
</commit_message>
<xml_diff>
--- a/skills/stolen-bell-tipout/forms/CashOut_Form.xlsx
+++ b/skills/stolen-bell-tipout/forms/CashOut_Form.xlsx
@@ -698,7 +698,7 @@
         </is>
       </c>
       <c r="B20" s="30">
-        <f>IF((COUNTIFS($E$23:$E$25,"Host",$C$23:$C$25,"&gt;0")&gt;0)+(COUNTIFS($E$23:$E$25,"Barback",$C$23:$C$25,"&gt;0")&gt;0)+(COUNTIFS($E$23:$E$25,"Busser",$C$23:$C$25,"&gt;0")&gt;0)&gt;=2,0.0225,IF((COUNTIFS($E$23:$E$25,"Host",$C$23:$C$25,"&gt;0")&gt;0)+(COUNTIFS($E$23:$E$25,"Barback",$C$23:$C$25,"&gt;0")&gt;0)+(COUNTIFS($E$23:$E$25,"Busser",$C$23:$C$25,"&gt;0")&gt;0)=1,0.015,0))</f>
+        <f>IF((COUNTIFS($E$23:$E$25,"Host",$C$23:$C$25,"&gt;0")&gt;0)+(COUNTIFS($E$23:$E$25,"Barback",$C$23:$C$25,"&gt;0")&gt;0)+(COUNTIFS($E$23:$E$25,"Busser",$C$23:$C$25,"&gt;0")&gt;0)+(COUNTIFS($E$23:$E$25,"Runner",$C$23:$C$25,"&gt;0")&gt;0)&gt;=2,0.0225,IF((COUNTIFS($E$23:$E$25,"Host",$C$23:$C$25,"&gt;0")&gt;0)+(COUNTIFS($E$23:$E$25,"Barback",$C$23:$C$25,"&gt;0")&gt;0)+(COUNTIFS($E$23:$E$25,"Busser",$C$23:$C$25,"&gt;0")&gt;0)+(COUNTIFS($E$23:$E$25,"Runner",$C$23:$C$25,"&gt;0")&gt;0)=1,0.015,0))</f>
         <v/>
       </c>
     </row>
@@ -1057,7 +1057,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation sqref="E23:E25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Host,Barback,Busser"</formula1>
+      <formula1>"Host,Barback,Busser,Runner"</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -1250,7 +1250,7 @@
         </is>
       </c>
       <c r="B20" s="30">
-        <f>IF((COUNTIFS($E$23:$E$25,"Host",$C$23:$C$25,"&gt;0")&gt;0)+(COUNTIFS($E$23:$E$25,"Barback",$C$23:$C$25,"&gt;0")&gt;0)+(COUNTIFS($E$23:$E$25,"Busser",$C$23:$C$25,"&gt;0")&gt;0)&gt;=2,0.0225,IF((COUNTIFS($E$23:$E$25,"Host",$C$23:$C$25,"&gt;0")&gt;0)+(COUNTIFS($E$23:$E$25,"Barback",$C$23:$C$25,"&gt;0")&gt;0)+(COUNTIFS($E$23:$E$25,"Busser",$C$23:$C$25,"&gt;0")&gt;0)=1,0.015,0))</f>
+        <f>IF((COUNTIFS($E$23:$E$25,"Host",$C$23:$C$25,"&gt;0")&gt;0)+(COUNTIFS($E$23:$E$25,"Barback",$C$23:$C$25,"&gt;0")&gt;0)+(COUNTIFS($E$23:$E$25,"Busser",$C$23:$C$25,"&gt;0")&gt;0)+(COUNTIFS($E$23:$E$25,"Runner",$C$23:$C$25,"&gt;0")&gt;0)&gt;=2,0.0225,IF((COUNTIFS($E$23:$E$25,"Host",$C$23:$C$25,"&gt;0")&gt;0)+(COUNTIFS($E$23:$E$25,"Barback",$C$23:$C$25,"&gt;0")&gt;0)+(COUNTIFS($E$23:$E$25,"Busser",$C$23:$C$25,"&gt;0")&gt;0)+(COUNTIFS($E$23:$E$25,"Runner",$C$23:$C$25,"&gt;0")&gt;0)=1,0.015,0))</f>
         <v/>
       </c>
     </row>
@@ -1647,7 +1647,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation sqref="E23:E25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Host,Barback,Busser"</formula1>
+      <formula1>"Host,Barback,Busser,Runner"</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>

<commit_message>
Cash Out form: write the hourly rate; show names as first name + last initial
- fill_cashout writes Hourly rate (ref) on each bar/server row (bar/server
  remainder / their total hours) so it shows without recalculation, and
  marks the workbook to recalculate fully when opened in Excel. Header
  restored to 'Hourly rate (ref)'.
- get_tipout_inputs names people 'First L.'; anyone whose short name
  would clash is shown in full (and with an ID if that clashes too).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015jcTPXYQVoMy2BAsKbkHbq
</commit_message>
<xml_diff>
--- a/skills/stolen-bell-tipout/forms/CashOut_Form.xlsx
+++ b/skills/stolen-bell-tipout/forms/CashOut_Form.xlsx
@@ -820,7 +820,7 @@
       </c>
       <c r="D29" s="39" t="inlineStr">
         <is>
-          <t>Hourly rate</t>
+          <t>Hourly rate (ref)</t>
         </is>
       </c>
       <c r="E29" s="39" t="inlineStr">
@@ -1392,7 +1392,7 @@
       </c>
       <c r="D29" s="39" t="inlineStr">
         <is>
-          <t>Hourly rate</t>
+          <t>Hourly rate (ref)</t>
         </is>
       </c>
       <c r="E29" s="39" t="inlineStr">

</xml_diff>